<commit_message>
docs(qa): combinar celdas de tópico (merge vertical) + más espacio en RESPUESTA para capturas
Ajuste pedido: columna TÓPICO combinada verticalmente por grupo (una celda por tópico,
centrada); columna RESPUESTA KOMFIA ensanchada (ancho 60) y alto de fila 78 para pegar
capturas, sin exagerar.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/KomfIA_Preguntas y Respuestas.xlsx
+++ b/docs/KomfIA_Preguntas y Respuestas.xlsx
@@ -64,7 +64,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -86,11 +86,44 @@
         <color rgb="00BFBFBF"/>
       </bottom>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00BFBFBF"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00BFBFBF"/>
+      </left>
+      <right style="thin">
+        <color rgb="00BFBFBF"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00BFBFBF"/>
+      </left>
+      <right style="thin">
+        <color rgb="00BFBFBF"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="00BFBFBF"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -100,7 +133,7 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -108,7 +141,8 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -478,11 +512,11 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
-    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
     <col width="6" customWidth="1" min="3" max="3"/>
-    <col width="52" customWidth="1" min="4" max="4"/>
-    <col width="42" customWidth="1" min="5" max="5"/>
-    <col width="66" customWidth="1" min="6" max="6"/>
+    <col width="50" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
+    <col width="62" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -527,7 +561,7 @@
         </is>
       </c>
     </row>
-    <row r="5">
+    <row r="5" ht="78" customHeight="1">
       <c r="B5" s="4" t="inlineStr">
         <is>
           <t>0. BASE / CONTEO</t>
@@ -548,7 +582,7 @@
         </is>
       </c>
     </row>
-    <row r="6">
+    <row r="6" ht="78" customHeight="1">
       <c r="B6" s="4" t="inlineStr">
         <is>
           <t>1. ÚLTIMO ANÁLISIS / CONDICIÓN</t>
@@ -569,7 +603,7 @@
         </is>
       </c>
     </row>
-    <row r="7">
+    <row r="7" ht="78" customHeight="1">
       <c r="B7" s="7" t="n"/>
       <c r="C7" s="5" t="n">
         <v>3</v>
@@ -586,7 +620,7 @@
         </is>
       </c>
     </row>
-    <row r="8">
+    <row r="8" ht="78" customHeight="1">
       <c r="B8" s="4" t="inlineStr">
         <is>
           <t>2. DIAGNÓSTICO (equipo)</t>
@@ -607,8 +641,8 @@
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="B9" s="7" t="n"/>
+    <row r="9" ht="78" customHeight="1">
+      <c r="B9" s="8" t="n"/>
       <c r="C9" s="5" t="n">
         <v>5</v>
       </c>
@@ -623,7 +657,7 @@
         <v/>
       </c>
     </row>
-    <row r="10">
+    <row r="10" ht="78" customHeight="1">
       <c r="B10" s="7" t="n"/>
       <c r="C10" s="5" t="n">
         <v>6</v>
@@ -640,7 +674,7 @@
         </is>
       </c>
     </row>
-    <row r="11">
+    <row r="11" ht="78" customHeight="1">
       <c r="B11" s="4" t="inlineStr">
         <is>
           <t>3. TRIAGE / RANKING (universo)</t>
@@ -661,7 +695,7 @@
         </is>
       </c>
     </row>
-    <row r="12">
+    <row r="12" ht="78" customHeight="1">
       <c r="B12" s="7" t="n"/>
       <c r="C12" s="5" t="n">
         <v>8</v>
@@ -678,7 +712,7 @@
         </is>
       </c>
     </row>
-    <row r="13">
+    <row r="13" ht="78" customHeight="1">
       <c r="B13" s="4" t="inlineStr">
         <is>
           <t>4. TENDENCIAS</t>
@@ -699,8 +733,8 @@
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="B14" s="7" t="n"/>
+    <row r="14" ht="78" customHeight="1">
+      <c r="B14" s="8" t="n"/>
       <c r="C14" s="5" t="n">
         <v>10</v>
       </c>
@@ -716,8 +750,8 @@
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="B15" s="7" t="n"/>
+    <row r="15" ht="78" customHeight="1">
+      <c r="B15" s="8" t="n"/>
       <c r="C15" s="5" t="n">
         <v>11</v>
       </c>
@@ -733,8 +767,8 @@
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="B16" s="7" t="n"/>
+    <row r="16" ht="78" customHeight="1">
+      <c r="B16" s="8" t="n"/>
       <c r="C16" s="5" t="n">
         <v>12</v>
       </c>
@@ -750,7 +784,7 @@
         </is>
       </c>
     </row>
-    <row r="17">
+    <row r="17" ht="78" customHeight="1">
       <c r="B17" s="7" t="n"/>
       <c r="C17" s="5" t="n">
         <v>13</v>
@@ -767,7 +801,7 @@
         </is>
       </c>
     </row>
-    <row r="18">
+    <row r="18" ht="78" customHeight="1">
       <c r="B18" s="4" t="inlineStr">
         <is>
           <t>5. BARRIDO / OBSERVADOS (flota)</t>
@@ -788,8 +822,8 @@
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="B19" s="7" t="n"/>
+    <row r="19" ht="78" customHeight="1">
+      <c r="B19" s="8" t="n"/>
       <c r="C19" s="5" t="n">
         <v>15</v>
       </c>
@@ -805,8 +839,8 @@
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="B20" s="7" t="n"/>
+    <row r="20" ht="78" customHeight="1">
+      <c r="B20" s="8" t="n"/>
       <c r="C20" s="5" t="n">
         <v>16</v>
       </c>
@@ -822,7 +856,7 @@
         </is>
       </c>
     </row>
-    <row r="21">
+    <row r="21" ht="78" customHeight="1">
       <c r="B21" s="7" t="n"/>
       <c r="C21" s="5" t="n">
         <v>17</v>
@@ -839,7 +873,7 @@
         </is>
       </c>
     </row>
-    <row r="22">
+    <row r="22" ht="78" customHeight="1">
       <c r="B22" s="4" t="inlineStr">
         <is>
           <t>6. HISTORIAL</t>
@@ -860,8 +894,8 @@
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="B23" s="7" t="n"/>
+    <row r="23" ht="78" customHeight="1">
+      <c r="B23" s="8" t="n"/>
       <c r="C23" s="5" t="n">
         <v>19</v>
       </c>
@@ -877,8 +911,8 @@
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="B24" s="7" t="n"/>
+    <row r="24" ht="78" customHeight="1">
+      <c r="B24" s="8" t="n"/>
       <c r="C24" s="5" t="n">
         <v>20</v>
       </c>
@@ -894,8 +928,8 @@
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="B25" s="7" t="n"/>
+    <row r="25" ht="78" customHeight="1">
+      <c r="B25" s="8" t="n"/>
       <c r="C25" s="5" t="n">
         <v>21</v>
       </c>
@@ -911,7 +945,7 @@
         </is>
       </c>
     </row>
-    <row r="26">
+    <row r="26" ht="78" customHeight="1">
       <c r="B26" s="7" t="n"/>
       <c r="C26" s="5" t="n">
         <v>22</v>
@@ -928,7 +962,7 @@
         </is>
       </c>
     </row>
-    <row r="27">
+    <row r="27" ht="78" customHeight="1">
       <c r="B27" s="4" t="inlineStr">
         <is>
           <t>7. CONTINUIDAD</t>
@@ -949,8 +983,8 @@
         </is>
       </c>
     </row>
-    <row r="28">
-      <c r="B28" s="7" t="n"/>
+    <row r="28" ht="78" customHeight="1">
+      <c r="B28" s="8" t="n"/>
       <c r="C28" s="5" t="n">
         <v>24</v>
       </c>
@@ -966,8 +1000,8 @@
         </is>
       </c>
     </row>
-    <row r="29">
-      <c r="B29" s="7" t="n"/>
+    <row r="29" ht="78" customHeight="1">
+      <c r="B29" s="8" t="n"/>
       <c r="C29" s="5" t="n">
         <v>25</v>
       </c>
@@ -983,7 +1017,7 @@
         </is>
       </c>
     </row>
-    <row r="30">
+    <row r="30" ht="78" customHeight="1">
       <c r="B30" s="7" t="n"/>
       <c r="C30" s="5" t="n">
         <v>26</v>
@@ -1000,7 +1034,7 @@
         </is>
       </c>
     </row>
-    <row r="31">
+    <row r="31" ht="78" customHeight="1">
       <c r="B31" s="4" t="inlineStr">
         <is>
           <t>8. LÍMITE / BORDE</t>
@@ -1021,7 +1055,7 @@
         </is>
       </c>
     </row>
-    <row r="32">
+    <row r="32" ht="78" customHeight="1">
       <c r="B32" s="7" t="n"/>
       <c r="C32" s="5" t="n">
         <v>28</v>
@@ -1038,7 +1072,7 @@
         </is>
       </c>
     </row>
-    <row r="33">
+    <row r="33" ht="78" customHeight="1">
       <c r="B33" s="4" t="inlineStr">
         <is>
           <t>9. NUEVO (gerencia 07-2026)</t>
@@ -1059,8 +1093,8 @@
         </is>
       </c>
     </row>
-    <row r="34">
-      <c r="B34" s="7" t="n"/>
+    <row r="34" ht="78" customHeight="1">
+      <c r="B34" s="8" t="n"/>
       <c r="C34" s="5" t="n">
         <v>30</v>
       </c>
@@ -1076,8 +1110,8 @@
         </is>
       </c>
     </row>
-    <row r="35">
-      <c r="B35" s="7" t="n"/>
+    <row r="35" ht="78" customHeight="1">
+      <c r="B35" s="8" t="n"/>
       <c r="C35" s="5" t="n">
         <v>31</v>
       </c>
@@ -1093,7 +1127,7 @@
         </is>
       </c>
     </row>
-    <row r="36">
+    <row r="36" ht="78" customHeight="1">
       <c r="B36" s="7" t="n"/>
       <c r="C36" s="5" t="n">
         <v>32</v>
@@ -1111,9 +1145,18 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="11">
     <mergeCell ref="B2:F2"/>
+    <mergeCell ref="B18:B21"/>
+    <mergeCell ref="B11:B12"/>
+    <mergeCell ref="B13:B17"/>
+    <mergeCell ref="B8:B10"/>
     <mergeCell ref="B1:F1"/>
+    <mergeCell ref="B22:B26"/>
+    <mergeCell ref="B33:B36"/>
+    <mergeCell ref="B27:B30"/>
+    <mergeCell ref="B6:B7"/>
+    <mergeCell ref="B31:B32"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
fix(qa): eliminar celda que Excel tomaba como fórmula (evita el diálogo de reparación)
Una celda de RESULTADO ESPERADO empezaba con '=' → openpyxl la escribía como <f> (fórmula)
→ Excel la reparaba/quitaba al abrir. Reescrito el inicio ('= MISMA…' → 'Igual a la tabla…')
y añadido guardián: ninguna celda de texto puede arrancar con =,+,@. Verificado: 0 celdas
fórmula. Merges de tópico y formato intactos.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/KomfIA_Preguntas y Respuestas.xlsx
+++ b/docs/KomfIA_Preguntas y Respuestas.xlsx
@@ -652,9 +652,10 @@
         </is>
       </c>
       <c r="E9" s="6" t="inlineStr"/>
-      <c r="F9" s="6">
-        <f> MISMA tabla ancha que diagnóstico. '2 de 6' (MT LH + Sist. Hidr. críticos). Valida equivalencia último-general = diagnóstico.</f>
-        <v/>
+      <c r="F9" s="6" t="inlineStr">
+        <is>
+          <t>Igual a la tabla ancha del diagnóstico. '2 de 6' (MT LH + Sist. Hidr. críticos). Valida la equivalencia último-general = diagnóstico.</t>
+        </is>
       </c>
     </row>
     <row r="10" ht="78" customHeight="1">

</xml_diff>